<commit_message>
Trying to speed up 1a_import_Busch.
</commit_message>
<xml_diff>
--- a/Output/chapman_growth_example.xlsx
+++ b/Output/chapman_growth_example.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t xml:space="preserve">How does the Chapman growth function work?</t>
   </si>
@@ -28,15 +28,28 @@
     <t xml:space="preserve">A</t>
   </si>
   <si>
+    <t xml:space="preserve">Limit of growth</t>
+  </si>
+  <si>
     <t xml:space="preserve">k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% rate of growth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Period</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cumulative growth</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="General"/>
+    <numFmt numFmtId="165" formatCode="#,##0.00"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -68,20 +81,41 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE6E6E6"/>
+        <bgColor rgb="FFFFFFCC"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="hair">
+        <color rgb="FFA0A0A0"/>
+      </left>
+      <right style="hair">
+        <color rgb="FFA0A0A0"/>
+      </right>
+      <top style="hair">
+        <color rgb="FFA0A0A0"/>
+      </top>
+      <bottom style="hair">
+        <color rgb="FFA0A0A0"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -110,12 +144,20 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -131,7 +173,7 @@
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
-      <rgbColor rgb="FFFFFFFF"/>
+      <rgbColor rgb="FFE6E6E6"/>
       <rgbColor rgb="FFFF0000"/>
       <rgbColor rgb="FF00FF00"/>
       <rgbColor rgb="FF0000FF"/>
@@ -177,7 +219,7 @@
       <rgbColor rgb="FFFF9900"/>
       <rgbColor rgb="FFFF420E"/>
       <rgbColor rgb="FF666699"/>
-      <rgbColor rgb="FF969696"/>
+      <rgbColor rgb="FFA0A0A0"/>
       <rgbColor rgb="FF003366"/>
       <rgbColor rgb="FF339966"/>
       <rgbColor rgb="FF003300"/>
@@ -198,6 +240,17 @@
   <c:chart>
     <c:autoTitleDeleted val="1"/>
     <c:plotArea>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.0595736700631369"/>
+          <c:y val="0.0419584305879738"/>
+          <c:w val="0.892292304807151"/>
+          <c:h val="0.866177614760476"/>
+        </c:manualLayout>
+      </c:layout>
       <c:lineChart>
         <c:grouping val="standard"/>
         <c:varyColors val="0"/>
@@ -265,90 +318,90 @@
           </c:dLbls>
           <c:val>
             <c:numRef>
-              <c:f>Chapman!$B$4:$B$30</c:f>
+              <c:f>Chapman!$B$7:$B$33</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>#,##0.00</c:formatCode>
                 <c:ptCount val="27"/>
                 <c:pt idx="0">
-                  <c:v>0.2</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1.31434159518702</c:v>
+                  <c:v>15.9830560357491</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>4.34755488183772</c:v>
+                  <c:v>29.9058028966204</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>8.14283758896597</c:v>
+                  <c:v>36.1161846176375</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>12.1295435904085</c:v>
+                  <c:v>38.5481673940174</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>15.9830560357491</c:v>
+                  <c:v>39.4627802372637</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>19.5331811786003</c:v>
+                  <c:v>39.8019455943608</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>22.7046453896802</c:v>
+                  <c:v>39.9270827039044</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>25.4787667195622</c:v>
+                  <c:v>39.9731674911748</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>27.8690378401648</c:v>
+                  <c:v>39.9901278248723</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>29.9058028966204</c:v>
+                  <c:v>39.9963680880652</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>31.626840927136</c:v>
+                  <c:v>39.9986638750947</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>33.0717536188078</c:v>
+                  <c:v>39.9995084645218</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>34.2787763196837</c:v>
+                  <c:v>39.9998191738518</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>35.2831095386419</c:v>
+                  <c:v>39.9999334777301</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>36.1161846176375</c:v>
+                  <c:v>39.9999755278181</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>36.8054859726577</c:v>
+                  <c:v>39.9999909971865</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>37.3746894090877</c:v>
+                  <c:v>39.9999966880499</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>37.8439656365517</c:v>
+                  <c:v>39.9999987816016</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>38.2303563088444</c:v>
+                  <c:v>39.9999995517763</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>38.5481673940174</c:v>
+                  <c:v>39.9999998351077</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>38.8093485473289</c:v>
+                  <c:v>39.9999999393395</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>39.0238421307584</c:v>
+                  <c:v>39.9999999776843</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>39.1998947165028</c:v>
+                  <c:v>39.9999999917905</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>39.344329385538</c:v>
+                  <c:v>39.9999999969799</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>39.4627802372637</c:v>
+                  <c:v>39.999999998889</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>39.5598921456595</c:v>
+                  <c:v>39.9999999995913</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -419,90 +472,90 @@
           </c:dLbls>
           <c:val>
             <c:numRef>
-              <c:f>Chapman!$C$4:$C$30</c:f>
+              <c:f>Chapman!$C$7:$C$33</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>#,##0.00</c:formatCode>
                 <c:ptCount val="27"/>
                 <c:pt idx="0">
-                  <c:v>0.1</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.606764937360043</c:v>
+                  <c:v>0.00396023233676776</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>4.97242303935513</c:v>
+                  <c:v>0.0156837015525043</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>12.4118994425582</c:v>
+                  <c:v>0.0349386594892943</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>19.7505023406946</c:v>
+                  <c:v>0.0614987232795747</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>25.4569108611625</c:v>
+                  <c:v>0.0951427613812622</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>29.4600992999427</c:v>
+                  <c:v>0.135654781946404</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>32.1654038936808</c:v>
+                  <c:v>0.182823823476374</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>33.9850968854884</c:v>
+                  <c:v>0.236443847717591</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>35.2229054164409</c:v>
+                  <c:v>0.296313634752626</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>36.080374610919</c:v>
+                  <c:v>0.362236680242509</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>36.6866507468586</c:v>
+                  <c:v>0.43402109477688</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>37.1240822440535</c:v>
+                  <c:v>0.511479505289536</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>37.4456749683432</c:v>
+                  <c:v>0.594428958497746</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>37.6861109574727</c:v>
+                  <c:v>0.682690826324553</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>37.8685295066025</c:v>
+                  <c:v>0.77609071326409</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>38.0086887223511</c:v>
+                  <c:v>0.87445836565073</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>38.1175406540663</c:v>
+                  <c:v>0.977627582793694</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>38.2028469867573</c:v>
+                  <c:v>1.08543612993948</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>38.2702097531847</c:v>
+                  <c:v>1.19772565302525</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>38.323740716831</c:v>
+                  <c:v>1.31434159518702</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>38.3665041045352</c:v>
+                  <c:v>1.4351331149873</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>38.4008148013581</c:v>
+                  <c:v>1.55995300632738</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>38.4284428020482</c:v>
+                  <c:v>1.68865762001032</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>38.4507558286248</c:v>
+                  <c:v>1.82110678692136</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>38.468820477177</c:v>
+                  <c:v>1.95716374279295</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>38.4834750933703</c:v>
+                  <c:v>2.09669505452247</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -517,11 +570,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="48286105"/>
-        <c:axId val="25492126"/>
+        <c:axId val="31858931"/>
+        <c:axId val="70442787"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="48286105"/>
+        <c:axId val="31858931"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -553,7 +606,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="25492126"/>
+        <c:crossAx val="70442787"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -561,21 +614,12 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="25492126"/>
+        <c:axId val="70442787"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln w="0">
-              <a:solidFill>
-                <a:srgbClr val="B3B3B3"/>
-              </a:solidFill>
-            </a:ln>
-          </c:spPr>
-        </c:majorGridlines>
         <c:numFmt formatCode="General" sourceLinked="0"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
@@ -602,7 +646,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="48286105"/>
+        <c:crossAx val="31858931"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -617,6 +661,16 @@
     </c:plotArea>
     <c:legend>
       <c:legendPos val="r"/>
+      <c:layout>
+        <c:manualLayout>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.602237919609927"/>
+          <c:y val="0.442036234300322"/>
+          <c:w val="0.166406201162718"/>
+          <c:h val="0.191397132377459"/>
+        </c:manualLayout>
+      </c:layout>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -664,9 +718,11 @@
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="419">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor"/>
+    <cs:lineWidthScale>1</cs:lineWidthScale>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor"/>
+    <a:defRPr sz="1800" b="0"/>
   </cs:axisTitle>
   <cs:categoryAxis>
     <cs:lnRef idx="0"/>
@@ -874,16 +930,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>3960</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>74160</xdr:rowOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>569880</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>189000</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>13</xdr:col>
-      <xdr:colOff>402480</xdr:colOff>
-      <xdr:row>21</xdr:row>
-      <xdr:rowOff>74880</xdr:rowOff>
+      <xdr:colOff>372600</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>189360</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -891,8 +947,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="2386440" y="836280"/>
-        <a:ext cx="5759280" cy="3239280"/>
+        <a:off x="2356920" y="2284560"/>
+        <a:ext cx="5758920" cy="3238920"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -1085,17 +1141,17 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C30"/>
+  <dimension ref="A1:D33"/>
   <sheetFormatPr defaultColWidth="8.453125" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
       <c r="B3" s="1" t="n">
@@ -1104,354 +1160,387 @@
       <c r="C3" s="1" t="n">
         <v>40</v>
       </c>
+      <c r="D3" s="0" t="s">
+        <v>2</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="s">
-        <v>2</v>
+      <c r="A4" s="2" t="s">
+        <v>3</v>
       </c>
       <c r="B4" s="1" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="C4" s="1" t="n">
-        <v>0.1</v>
+        <v>0.01</v>
+      </c>
+      <c r="D4" s="0" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="B5" s="1" t="n">
-        <f aca="false">B$3*(1-EXP(-B$4*A5))^2</f>
-        <v>1.31434159518702</v>
-      </c>
-      <c r="C5" s="1" t="n">
-        <f aca="false">C$3*(1-EXP(-C$4*B5))^2</f>
-        <v>0.606764937360043</v>
-      </c>
+      <c r="A5" s="1"/>
+      <c r="B5" s="1"/>
+      <c r="C5" s="1"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="B6" s="1" t="n">
-        <f aca="false">$B$3*(1-EXP(-$B$4*A6))^2</f>
-        <v>4.34755488183772</v>
-      </c>
-      <c r="C6" s="1" t="n">
-        <f aca="false">C$3*(1-EXP(-C$4*B6))^2</f>
-        <v>4.97242303935513</v>
-      </c>
+      <c r="A6" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" s="1"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="n">
-        <v>3</v>
-      </c>
-      <c r="B7" s="1" t="n">
-        <f aca="false">$B$3*(1-EXP(-$B$4*A7))^2</f>
-        <v>8.14283758896597</v>
-      </c>
-      <c r="C7" s="1" t="n">
-        <f aca="false">C$3*(1-EXP(-C$4*B7))^2</f>
-        <v>12.4118994425582</v>
+        <v>0</v>
+      </c>
+      <c r="B7" s="3" t="n">
+        <f aca="false">B$3*(1-EXP(-B$4*$A7))^2</f>
+        <v>0</v>
+      </c>
+      <c r="C7" s="3" t="n">
+        <f aca="false">C$3*(1-EXP(-C$4*$A7))^2</f>
+        <v>0</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="n">
-        <v>4</v>
-      </c>
-      <c r="B8" s="1" t="n">
-        <f aca="false">$B$3*(1-EXP(-$B$4*A8))^2</f>
-        <v>12.1295435904085</v>
-      </c>
-      <c r="C8" s="1" t="n">
-        <f aca="false">C$3*(1-EXP(-C$4*B8))^2</f>
-        <v>19.7505023406946</v>
+        <v>1</v>
+      </c>
+      <c r="B8" s="3" t="n">
+        <f aca="false">B$3*(1-EXP(-B$4*$A8))^2</f>
+        <v>15.9830560357491</v>
+      </c>
+      <c r="C8" s="3" t="n">
+        <f aca="false">C$3*(1-EXP(-C$4*$A8))^2</f>
+        <v>0.00396023233676776</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="n">
-        <v>5</v>
-      </c>
-      <c r="B9" s="1" t="n">
-        <f aca="false">$B$3*(1-EXP(-$B$4*A9))^2</f>
-        <v>15.9830560357491</v>
-      </c>
-      <c r="C9" s="1" t="n">
-        <f aca="false">C$3*(1-EXP(-C$4*B9))^2</f>
-        <v>25.4569108611625</v>
+        <v>2</v>
+      </c>
+      <c r="B9" s="3" t="n">
+        <f aca="false">B$3*(1-EXP(-B$4*$A9))^2</f>
+        <v>29.9058028966204</v>
+      </c>
+      <c r="C9" s="3" t="n">
+        <f aca="false">C$3*(1-EXP(-C$4*$A9))^2</f>
+        <v>0.0156837015525043</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="n">
-        <v>6</v>
-      </c>
-      <c r="B10" s="1" t="n">
-        <f aca="false">$B$3*(1-EXP(-$B$4*A10))^2</f>
-        <v>19.5331811786003</v>
-      </c>
-      <c r="C10" s="1" t="n">
-        <f aca="false">C$3*(1-EXP(-C$4*B10))^2</f>
-        <v>29.4600992999427</v>
+        <v>3</v>
+      </c>
+      <c r="B10" s="3" t="n">
+        <f aca="false">B$3*(1-EXP(-B$4*$A10))^2</f>
+        <v>36.1161846176375</v>
+      </c>
+      <c r="C10" s="3" t="n">
+        <f aca="false">C$3*(1-EXP(-C$4*$A10))^2</f>
+        <v>0.0349386594892943</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="n">
-        <v>7</v>
-      </c>
-      <c r="B11" s="1" t="n">
-        <f aca="false">$B$3*(1-EXP(-$B$4*A11))^2</f>
-        <v>22.7046453896802</v>
-      </c>
-      <c r="C11" s="1" t="n">
-        <f aca="false">C$3*(1-EXP(-C$4*B11))^2</f>
-        <v>32.1654038936808</v>
+        <v>4</v>
+      </c>
+      <c r="B11" s="3" t="n">
+        <f aca="false">B$3*(1-EXP(-B$4*$A11))^2</f>
+        <v>38.5481673940174</v>
+      </c>
+      <c r="C11" s="3" t="n">
+        <f aca="false">C$3*(1-EXP(-C$4*$A11))^2</f>
+        <v>0.0614987232795747</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="n">
-        <v>8</v>
-      </c>
-      <c r="B12" s="1" t="n">
-        <f aca="false">$B$3*(1-EXP(-$B$4*A12))^2</f>
-        <v>25.4787667195622</v>
-      </c>
-      <c r="C12" s="1" t="n">
-        <f aca="false">C$3*(1-EXP(-C$4*B12))^2</f>
-        <v>33.9850968854884</v>
+        <v>5</v>
+      </c>
+      <c r="B12" s="3" t="n">
+        <f aca="false">B$3*(1-EXP(-B$4*$A12))^2</f>
+        <v>39.4627802372637</v>
+      </c>
+      <c r="C12" s="3" t="n">
+        <f aca="false">C$3*(1-EXP(-C$4*$A12))^2</f>
+        <v>0.0951427613812622</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="n">
-        <v>9</v>
-      </c>
-      <c r="B13" s="1" t="n">
-        <f aca="false">$B$3*(1-EXP(-$B$4*A13))^2</f>
-        <v>27.8690378401648</v>
-      </c>
-      <c r="C13" s="1" t="n">
-        <f aca="false">C$3*(1-EXP(-C$4*B13))^2</f>
-        <v>35.2229054164409</v>
+        <v>6</v>
+      </c>
+      <c r="B13" s="3" t="n">
+        <f aca="false">B$3*(1-EXP(-B$4*$A13))^2</f>
+        <v>39.8019455943608</v>
+      </c>
+      <c r="C13" s="3" t="n">
+        <f aca="false">C$3*(1-EXP(-C$4*$A13))^2</f>
+        <v>0.135654781946404</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="n">
-        <v>10</v>
-      </c>
-      <c r="B14" s="1" t="n">
-        <f aca="false">$B$3*(1-EXP(-$B$4*A14))^2</f>
-        <v>29.9058028966204</v>
-      </c>
-      <c r="C14" s="1" t="n">
-        <f aca="false">C$3*(1-EXP(-C$4*B14))^2</f>
-        <v>36.080374610919</v>
+        <v>7</v>
+      </c>
+      <c r="B14" s="3" t="n">
+        <f aca="false">B$3*(1-EXP(-B$4*$A14))^2</f>
+        <v>39.9270827039044</v>
+      </c>
+      <c r="C14" s="3" t="n">
+        <f aca="false">C$3*(1-EXP(-C$4*$A14))^2</f>
+        <v>0.182823823476374</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="n">
-        <v>11</v>
-      </c>
-      <c r="B15" s="1" t="n">
-        <f aca="false">$B$3*(1-EXP(-$B$4*A15))^2</f>
-        <v>31.626840927136</v>
-      </c>
-      <c r="C15" s="1" t="n">
-        <f aca="false">C$3*(1-EXP(-C$4*B15))^2</f>
-        <v>36.6866507468586</v>
+        <v>8</v>
+      </c>
+      <c r="B15" s="3" t="n">
+        <f aca="false">B$3*(1-EXP(-B$4*$A15))^2</f>
+        <v>39.9731674911748</v>
+      </c>
+      <c r="C15" s="3" t="n">
+        <f aca="false">C$3*(1-EXP(-C$4*$A15))^2</f>
+        <v>0.236443847717591</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="n">
-        <v>12</v>
-      </c>
-      <c r="B16" s="1" t="n">
-        <f aca="false">$B$3*(1-EXP(-$B$4*A16))^2</f>
-        <v>33.0717536188078</v>
-      </c>
-      <c r="C16" s="1" t="n">
-        <f aca="false">C$3*(1-EXP(-C$4*B16))^2</f>
-        <v>37.1240822440535</v>
+        <v>9</v>
+      </c>
+      <c r="B16" s="3" t="n">
+        <f aca="false">B$3*(1-EXP(-B$4*$A16))^2</f>
+        <v>39.9901278248723</v>
+      </c>
+      <c r="C16" s="3" t="n">
+        <f aca="false">C$3*(1-EXP(-C$4*$A16))^2</f>
+        <v>0.296313634752626</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="n">
-        <v>13</v>
-      </c>
-      <c r="B17" s="1" t="n">
-        <f aca="false">$B$3*(1-EXP(-$B$4*A17))^2</f>
-        <v>34.2787763196837</v>
-      </c>
-      <c r="C17" s="1" t="n">
-        <f aca="false">C$3*(1-EXP(-C$4*B17))^2</f>
-        <v>37.4456749683432</v>
+        <v>10</v>
+      </c>
+      <c r="B17" s="3" t="n">
+        <f aca="false">B$3*(1-EXP(-B$4*$A17))^2</f>
+        <v>39.9963680880652</v>
+      </c>
+      <c r="C17" s="3" t="n">
+        <f aca="false">C$3*(1-EXP(-C$4*$A17))^2</f>
+        <v>0.362236680242509</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="n">
-        <v>14</v>
-      </c>
-      <c r="B18" s="1" t="n">
-        <f aca="false">$B$3*(1-EXP(-$B$4*A18))^2</f>
-        <v>35.2831095386419</v>
-      </c>
-      <c r="C18" s="1" t="n">
-        <f aca="false">C$3*(1-EXP(-C$4*B18))^2</f>
-        <v>37.6861109574727</v>
+        <v>11</v>
+      </c>
+      <c r="B18" s="3" t="n">
+        <f aca="false">B$3*(1-EXP(-B$4*$A18))^2</f>
+        <v>39.9986638750947</v>
+      </c>
+      <c r="C18" s="3" t="n">
+        <f aca="false">C$3*(1-EXP(-C$4*$A18))^2</f>
+        <v>0.43402109477688</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="n">
-        <v>15</v>
-      </c>
-      <c r="B19" s="1" t="n">
-        <f aca="false">$B$3*(1-EXP(-$B$4*A19))^2</f>
-        <v>36.1161846176375</v>
-      </c>
-      <c r="C19" s="1" t="n">
-        <f aca="false">C$3*(1-EXP(-C$4*B19))^2</f>
-        <v>37.8685295066025</v>
+        <v>12</v>
+      </c>
+      <c r="B19" s="3" t="n">
+        <f aca="false">B$3*(1-EXP(-B$4*$A19))^2</f>
+        <v>39.9995084645218</v>
+      </c>
+      <c r="C19" s="3" t="n">
+        <f aca="false">C$3*(1-EXP(-C$4*$A19))^2</f>
+        <v>0.511479505289536</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="n">
-        <v>16</v>
-      </c>
-      <c r="B20" s="1" t="n">
-        <f aca="false">$B$3*(1-EXP(-$B$4*A20))^2</f>
-        <v>36.8054859726577</v>
-      </c>
-      <c r="C20" s="1" t="n">
-        <f aca="false">C$3*(1-EXP(-C$4*B20))^2</f>
-        <v>38.0086887223511</v>
+        <v>13</v>
+      </c>
+      <c r="B20" s="3" t="n">
+        <f aca="false">B$3*(1-EXP(-B$4*$A20))^2</f>
+        <v>39.9998191738518</v>
+      </c>
+      <c r="C20" s="3" t="n">
+        <f aca="false">C$3*(1-EXP(-C$4*$A20))^2</f>
+        <v>0.594428958497746</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="n">
-        <v>17</v>
-      </c>
-      <c r="B21" s="1" t="n">
-        <f aca="false">$B$3*(1-EXP(-$B$4*A21))^2</f>
-        <v>37.3746894090877</v>
-      </c>
-      <c r="C21" s="1" t="n">
-        <f aca="false">C$3*(1-EXP(-C$4*B21))^2</f>
-        <v>38.1175406540663</v>
+        <v>14</v>
+      </c>
+      <c r="B21" s="3" t="n">
+        <f aca="false">B$3*(1-EXP(-B$4*$A21))^2</f>
+        <v>39.9999334777301</v>
+      </c>
+      <c r="C21" s="3" t="n">
+        <f aca="false">C$3*(1-EXP(-C$4*$A21))^2</f>
+        <v>0.682690826324553</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="n">
-        <v>18</v>
-      </c>
-      <c r="B22" s="1" t="n">
-        <f aca="false">$B$3*(1-EXP(-$B$4*A22))^2</f>
-        <v>37.8439656365517</v>
-      </c>
-      <c r="C22" s="1" t="n">
-        <f aca="false">C$3*(1-EXP(-C$4*B22))^2</f>
-        <v>38.2028469867573</v>
+        <v>15</v>
+      </c>
+      <c r="B22" s="3" t="n">
+        <f aca="false">B$3*(1-EXP(-B$4*$A22))^2</f>
+        <v>39.9999755278181</v>
+      </c>
+      <c r="C22" s="3" t="n">
+        <f aca="false">C$3*(1-EXP(-C$4*$A22))^2</f>
+        <v>0.77609071326409</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="n">
-        <v>19</v>
-      </c>
-      <c r="B23" s="1" t="n">
-        <f aca="false">$B$3*(1-EXP(-$B$4*A23))^2</f>
-        <v>38.2303563088444</v>
-      </c>
-      <c r="C23" s="1" t="n">
-        <f aca="false">C$3*(1-EXP(-C$4*B23))^2</f>
-        <v>38.2702097531847</v>
+        <v>16</v>
+      </c>
+      <c r="B23" s="3" t="n">
+        <f aca="false">B$3*(1-EXP(-B$4*$A23))^2</f>
+        <v>39.9999909971865</v>
+      </c>
+      <c r="C23" s="3" t="n">
+        <f aca="false">C$3*(1-EXP(-C$4*$A23))^2</f>
+        <v>0.87445836565073</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="n">
-        <v>20</v>
-      </c>
-      <c r="B24" s="1" t="n">
-        <f aca="false">$B$3*(1-EXP(-$B$4*A24))^2</f>
-        <v>38.5481673940174</v>
-      </c>
-      <c r="C24" s="1" t="n">
-        <f aca="false">C$3*(1-EXP(-C$4*B24))^2</f>
-        <v>38.323740716831</v>
+        <v>17</v>
+      </c>
+      <c r="B24" s="3" t="n">
+        <f aca="false">B$3*(1-EXP(-B$4*$A24))^2</f>
+        <v>39.9999966880499</v>
+      </c>
+      <c r="C24" s="3" t="n">
+        <f aca="false">C$3*(1-EXP(-C$4*$A24))^2</f>
+        <v>0.977627582793694</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="n">
-        <v>21</v>
-      </c>
-      <c r="B25" s="1" t="n">
-        <f aca="false">$B$3*(1-EXP(-$B$4*A25))^2</f>
-        <v>38.8093485473289</v>
-      </c>
-      <c r="C25" s="1" t="n">
-        <f aca="false">C$3*(1-EXP(-C$4*B25))^2</f>
-        <v>38.3665041045352</v>
+        <v>18</v>
+      </c>
+      <c r="B25" s="3" t="n">
+        <f aca="false">B$3*(1-EXP(-B$4*$A25))^2</f>
+        <v>39.9999987816016</v>
+      </c>
+      <c r="C25" s="3" t="n">
+        <f aca="false">C$3*(1-EXP(-C$4*$A25))^2</f>
+        <v>1.08543612993948</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="n">
-        <v>22</v>
-      </c>
-      <c r="B26" s="1" t="n">
-        <f aca="false">$B$3*(1-EXP(-$B$4*A26))^2</f>
-        <v>39.0238421307584</v>
-      </c>
-      <c r="C26" s="1" t="n">
-        <f aca="false">C$3*(1-EXP(-C$4*B26))^2</f>
-        <v>38.4008148013581</v>
+        <v>19</v>
+      </c>
+      <c r="B26" s="3" t="n">
+        <f aca="false">B$3*(1-EXP(-B$4*$A26))^2</f>
+        <v>39.9999995517763</v>
+      </c>
+      <c r="C26" s="3" t="n">
+        <f aca="false">C$3*(1-EXP(-C$4*$A26))^2</f>
+        <v>1.19772565302525</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="n">
-        <v>23</v>
-      </c>
-      <c r="B27" s="1" t="n">
-        <f aca="false">$B$3*(1-EXP(-$B$4*A27))^2</f>
-        <v>39.1998947165028</v>
-      </c>
-      <c r="C27" s="1" t="n">
-        <f aca="false">C$3*(1-EXP(-C$4*B27))^2</f>
-        <v>38.4284428020482</v>
+        <v>20</v>
+      </c>
+      <c r="B27" s="3" t="n">
+        <f aca="false">B$3*(1-EXP(-B$4*$A27))^2</f>
+        <v>39.9999998351077</v>
+      </c>
+      <c r="C27" s="3" t="n">
+        <f aca="false">C$3*(1-EXP(-C$4*$A27))^2</f>
+        <v>1.31434159518702</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="n">
-        <v>24</v>
-      </c>
-      <c r="B28" s="1" t="n">
-        <f aca="false">$B$3*(1-EXP(-$B$4*A28))^2</f>
-        <v>39.344329385538</v>
-      </c>
-      <c r="C28" s="1" t="n">
-        <f aca="false">C$3*(1-EXP(-C$4*B28))^2</f>
-        <v>38.4507558286248</v>
+        <v>21</v>
+      </c>
+      <c r="B28" s="3" t="n">
+        <f aca="false">B$3*(1-EXP(-B$4*$A28))^2</f>
+        <v>39.9999999393395</v>
+      </c>
+      <c r="C28" s="3" t="n">
+        <f aca="false">C$3*(1-EXP(-C$4*$A28))^2</f>
+        <v>1.4351331149873</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="n">
-        <v>25</v>
-      </c>
-      <c r="B29" s="1" t="n">
-        <f aca="false">$B$3*(1-EXP(-$B$4*A29))^2</f>
-        <v>39.4627802372637</v>
-      </c>
-      <c r="C29" s="1" t="n">
-        <f aca="false">C$3*(1-EXP(-C$4*B29))^2</f>
-        <v>38.468820477177</v>
+        <v>22</v>
+      </c>
+      <c r="B29" s="3" t="n">
+        <f aca="false">B$3*(1-EXP(-B$4*$A29))^2</f>
+        <v>39.9999999776843</v>
+      </c>
+      <c r="C29" s="3" t="n">
+        <f aca="false">C$3*(1-EXP(-C$4*$A29))^2</f>
+        <v>1.55995300632738</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="n">
+        <v>23</v>
+      </c>
+      <c r="B30" s="3" t="n">
+        <f aca="false">B$3*(1-EXP(-B$4*$A30))^2</f>
+        <v>39.9999999917905</v>
+      </c>
+      <c r="C30" s="3" t="n">
+        <f aca="false">C$3*(1-EXP(-C$4*$A30))^2</f>
+        <v>1.68865762001032</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="1" t="n">
+        <v>24</v>
+      </c>
+      <c r="B31" s="3" t="n">
+        <f aca="false">B$3*(1-EXP(-B$4*$A31))^2</f>
+        <v>39.9999999969799</v>
+      </c>
+      <c r="C31" s="3" t="n">
+        <f aca="false">C$3*(1-EXP(-C$4*$A31))^2</f>
+        <v>1.82110678692136</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="B32" s="3" t="n">
+        <f aca="false">B$3*(1-EXP(-B$4*$A32))^2</f>
+        <v>39.999999998889</v>
+      </c>
+      <c r="C32" s="3" t="n">
+        <f aca="false">C$3*(1-EXP(-C$4*$A32))^2</f>
+        <v>1.95716374279295</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="1" t="n">
         <v>26</v>
       </c>
-      <c r="B30" s="1" t="n">
-        <f aca="false">$B$3*(1-EXP(-$B$4*A30))^2</f>
-        <v>39.5598921456595</v>
-      </c>
-      <c r="C30" s="1" t="n">
-        <f aca="false">C$3*(1-EXP(-C$4*B30))^2</f>
-        <v>38.4834750933703</v>
+      <c r="B33" s="3" t="n">
+        <f aca="false">B$3*(1-EXP(-B$4*$A33))^2</f>
+        <v>39.9999999995913</v>
+      </c>
+      <c r="C33" s="3" t="n">
+        <f aca="false">C$3*(1-EXP(-C$4*$A33))^2</f>
+        <v>2.09669505452247</v>
       </c>
     </row>
   </sheetData>

</xml_diff>